<commit_message>
feat(qpcr): fix template TNF-a control variance (T1.3, M1)
</commit_message>
<xml_diff>
--- a/XSTARS_Templates.xlsx
+++ b/XSTARS_Templates.xlsx
@@ -1712,7 +1712,7 @@
         <v>12</v>
       </c>
       <c r="R11">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="S11">
         <v>24.5</v>
@@ -1726,7 +1726,7 @@
         <v>12</v>
       </c>
       <c r="R12">
-        <v>27.8</v>
+        <v>27.7</v>
       </c>
       <c r="S12">
         <v>24.2</v>

</xml_diff>